<commit_message>
feat: add shared CreditAtlas project and method register
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R02ed48f2d652431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R48dc05c407054231"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R854b1aa9d31648aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R2a1eef8d54234fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R08869772c5ce4a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Reb26adbaa3a94a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Rdd9c44a4c6604c26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="Rea581cc3384140d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -695,9 +695,11 @@
         <x:v>Tổng 26/50 tái tạo từ ledger; UI/docs không gọi 52% là D01; historical labels được giữ</x:v>
       </x:c>
       <x:c r="F18" s="17" t="str">
-        <x:v>Chưa bắt đầu</x:v>
-      </x:c>
-      <x:c r="G18" s="17" t="str"/>
+        <x:v>Đang làm</x:v>
+      </x:c>
+      <x:c r="G18" s="17" t="str">
+        <x:v>API/UI derives P1-P5 from the ledger; final local runtime review remains.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="68" customHeight="1">
       <x:c r="A19" s="10" t="str">
@@ -716,9 +718,11 @@
         <x:v>Mỗi source dùng bởi KPI có record; missing publication không thay bằng download date</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
-        <x:v>Chưa bắt đầu</x:v>
-      </x:c>
-      <x:c r="G19" s="17" t="str"/>
+        <x:v>Đang làm</x:v>
+      </x:c>
+      <x:c r="G19" s="17" t="str">
+        <x:v>24 priority source groups registered; remaining work is complete KPI-source coverage and receipt bindings.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="68" customHeight="1">
       <x:c r="A20" s="9" t="str">
@@ -737,9 +741,11 @@
         <x:v>Từng output số đi tới method/input; phân biệt publisher-imputed với app-imputed; không sửa frozen studies</x:v>
       </x:c>
       <x:c r="F20" s="17" t="str">
-        <x:v>Chưa bắt đầu</x:v>
-      </x:c>
-      <x:c r="G20" s="17" t="str"/>
+        <x:v>Đang làm</x:v>
+      </x:c>
+      <x:c r="G20" s="17" t="str">
+        <x:v>Seven provenance types and nine method cards registered; remaining work is output-level KPI/input lineage.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="68" customHeight="1">
       <x:c r="A21" s="10" t="str">
@@ -1211,7 +1217,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55217fd713144f35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdda63251514d05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2463,7 +2469,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0edc4bf022094e83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d351d8708340f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3122,7 +3128,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f4fd5a5b87d4ef4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2561f4547714159"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3273,7 +3279,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R050142cadcf4423e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a62bdb4297046a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: expand credit atlas source and next-step plan
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R08869772c5ce4a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Reb26adbaa3a94a7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Rdd9c44a4c6604c26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="Rea581cc3384140d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rdc86d48892a44e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R07ee048fa3ea4142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Reee1504894ef4979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R95ccc01db6c14e6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -197,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataInventory" displayName="DataInventory" ref="A5:G29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataInventory" displayName="DataInventory" ref="A5:G33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Nguồn"/>
     <x:tableColumn id="2" name="Số lượng"/>
@@ -451,7 +451,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Checkpoint 16/10/2026. Tỷ lệ của toàn P1–P5, không phải phần trăm D01 hoặc production readiness.</x:v>
+        <x:v>Checkpoint 17/10/2026. Tỷ lệ của toàn P1–P5, không phải phần trăm D01 hoặc production readiness.</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -701,7 +701,7 @@
         <x:v>API/UI derives P1-P5 from the ledger; final local runtime review remains.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="68" customHeight="1">
+    <x:row r="19" ht="66" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="str">
         <x:v>N02</x:v>
       </x:c>
@@ -709,19 +709,19 @@
         <x:v>Ngay / shared</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>Dataset registry cho source/release/grain/time/rights/use gates</x:v>
+        <x:v>Register 91 objects / 16 families; close source status, route parity, Excel and KPI-method links across 27 groups.</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
-        <x:v>Receipts đã có</x:v>
+        <x:v>Bound: HMDA 12, FHFA 9, LC/Bondora 5, HAMP 2, WDI 22, Sovereign 12; 16/27 groups bound, 11 open.</x:v>
       </x:c>
       <x:c r="E19" s="10" t="str">
-        <x:v>Mỗi source dùng bởi KPI có record; missing publication không thay bằng download date</x:v>
+        <x:v>27 groups statused; each KPI traces source → field → filter → formula → API/Excel; rights resolved/fenced; no unsupported estimates.</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
-        <x:v>Đang làm</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>24 priority source groups registered; remaining work is complete KPI-source coverage and receipt bindings.</x:v>
+        <x:v>WDI: 122,892 obs / 64,452 NULL. HAMP: 2018–21 activity gap. Sovereign: 4 editions, 515,678 missing, 72,509 zero, 68 count conflicts. Context data, not borrower PD.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="68" customHeight="1">
@@ -1217,7 +1217,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdda63251514d05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8af9fbf117f84f4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2469,7 +2469,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d351d8708340f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc68206f49ce14cfa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2598,7 +2598,7 @@
     </x:row>
     <x:row r="8" ht="50" customHeight="1">
       <x:c r="A8" s="9" t="str">
-        <x:v>LendingClub accepted</x:v>
+        <x:v>LendingClub accepted — Kaggle v3</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
         <x:v>2260701</x:v>
@@ -2607,13 +2607,13 @@
         <x:v>rows</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Full source archive</x:v>
+        <x:v>2007–2018Q4</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>P1 booked-loan research</x:v>
+        <x:v>P1 booked-loan cohort diagnostics</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>Feature timing/label maturity chưa qualify cho application model</x:v>
+        <x:v>151 fields; 33 missing/invalid issue dates; feature timing, label maturity and issuer rights unqualified</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
         <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/LENDINGCLUB_FULL_SOURCE_VI.md</x:v>
@@ -2621,7 +2621,7 @@
     </x:row>
     <x:row r="9" ht="50" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>LendingClub rejected</x:v>
+        <x:v>LendingClub rejected — Kaggle v3</x:v>
       </x:c>
       <x:c r="B9" s="19" t="n">
         <x:v>27648741</x:v>
@@ -2630,13 +2630,13 @@
         <x:v>rows</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Full source archive</x:v>
+        <x:v>2007–2018Q4</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>P1 application mix</x:v>
+        <x:v>P1 rejected-application population only</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>Không gộp với accepted để suy approval rate khi population chưa khớp</x:v>
+        <x:v>9 fields; 0 invalid application dates; no repayment outcome or compatible approval denominator</x:v>
       </x:c>
       <x:c r="G9" s="10" t="str">
         <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/LENDINGCLUB_FULL_SOURCE_VI.md</x:v>
@@ -2644,7 +2644,7 @@
     </x:row>
     <x:row r="10" ht="50" customHeight="1">
       <x:c r="A10" s="9" t="str">
-        <x:v>Bondora / Go &amp; Grow</x:v>
+        <x:v>Go &amp; Grow / Bondora Loan Dataset</x:v>
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:v>789144</x:v>
@@ -2653,16 +2653,16 @@
         <x:v>loans</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>2009–2026 snapshot</x:v>
+        <x:v>Issue dates 2009-02–2026-06</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>P1 temporal feasibility</x:v>
+        <x:v>P1 tri-state 12M label support</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>12M flags: 86.618 true / 520.246 false / 182.280 NULL</x:v>
+        <x:v>31 fields; 86,618 true / 520,246 false / 182,280 NULL; 10,860 proxy-mature NULL unresolved; retrieval/license unqualified</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
-        <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/BONDORA_PUBLIC_DATASET_RESEARCH_VI.md</x:v>
+        <x:v>https://goandgrow.eu/en/public-statistics/</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="50" customHeight="1">
@@ -2705,7 +2705,7 @@
         <x:v>Origination market context</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
-        <x:v>Đã audited; chưa app/Excel integration; VALUE1/2 tách biệt</x:v>
+        <x:v>App/API + query-scoped Excel đã tích hợp; browser visual và native Excel acceptance còn mở; VALUE1/2 tách biệt.</x:v>
       </x:c>
       <x:c r="G12" s="9" t="str">
         <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/FHFA_NMDB_ORIGINATION_OUTSTANDING_REVIEW_VI.md</x:v>
@@ -2738,18 +2738,20 @@
       <x:c r="A14" s="9" t="str">
         <x:v>HMDA 2018–2025</x:v>
       </x:c>
-      <x:c r="B14" s="18"/>
+      <x:c r="B14" s="18" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>release-specific rows</x:v>
+        <x:v>source release/file objects</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
-        <x:v>Three/One-Year, Snapshot/Dynamic</x:v>
+        <x:v>Activity 2018–2025; release freezes 2021–2026</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>D08 application/decision</x:v>
+        <x:v>D08 application/decision mix; descriptive denial analysis</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str">
-        <x:v>Không cộng releases; 2018 có 1.961 rows quarantine</x:v>
+        <x:v>9 LAR vintages + 3 QA/reference files. Row counts by LAR release are in the source register and overlap; 2018 has 1,961 quarantined rows. No repayment/default label.</x:v>
       </x:c>
       <x:c r="G14" s="9" t="str">
         <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/D01_PROGRESS_AND_DATA_PRIORITY_2026-10-16_VI.md</x:v>
@@ -2983,7 +2985,7 @@
         <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/STRUCTURED_ABS_SOURCE_WORKFLOW.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="50" customHeight="1">
+    <x:row r="25" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A25" s="10" t="str">
         <x:v>World Bank WDI</x:v>
       </x:c>
@@ -2991,19 +2993,19 @@
         <x:v>122892</x:v>
       </x:c>
       <x:c r="C25" s="10" t="str">
-        <x:v>annual observations</x:v>
+        <x:v>annual source observations; 7 indicators × 17,556 rows</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
-        <x:v>1960–2025, 7 indicators</x:v>
+        <x:v>Requested 1960–2025; WDI lastupdated 2026-10-08</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
-        <x:v>P4 country context</x:v>
+        <x:v>P4 country context; 217 economies + 49 returned aggregates; not borrower PD</x:v>
       </x:c>
       <x:c r="F25" s="10" t="str">
-        <x:v>217 economies / 49 aggregates riêng; không sovereign PD</x:v>
+        <x:v>64,452 source NULLs; NPL=2,357 known and capital=2,301 known; all aggregate NPL/capital rows NULL. No carry-forward. Third-party source terms need review.</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/COUNTRY_OBSERVATORY_WORKFLOW.md</x:v>
+        <x:v>https://github.com/susayold/credit-atlas/blob/main/docs/WORLD_BANK_WDI_DATA_REVIEW_VI.md</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="50" customHeight="1">
@@ -3014,22 +3016,22 @@
         <x:v>42519</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>edition-entity-year rows</x:v>
+        <x:v>Entity-year; 16 selected metrics / row</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>4 editions 2023–2026</x:v>
+        <x:v>Editions 2023–2026; reference years 1960–2025</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>P4 sovereign history</x:v>
+        <x:v>P4 sovereign-government default and revision context</x:v>
       </x:c>
       <x:c r="F26" s="9" t="str">
-        <x:v>Revisions/overlap; publication availability và calibrated stress chưa đủ</x:v>
+        <x:v>680,304 positions: 515,678 missing; 72,509 zero; 1,341 markers; 9,954 schema-absent; 68 count conflicts. Third-party rights review; not borrower PD/LGD.</x:v>
       </x:c>
       <x:c r="G26" s="9" t="str">
-        <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/SOVEREIGN_ARCHIVE_EDITIONS_VI.md</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="50" customHeight="1">
+        <x:v>https://github.com/susayold/credit-atlas/blob/main/docs/SOVEREIGN_ARCHIVE_DATA_REVIEW_VI.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="66" hidden="0" customHeight="1">
       <x:c r="A27" s="10" t="str">
         <x:v>Treasury HAMP</x:v>
       </x:c>
@@ -3037,19 +3039,19 @@
         <x:v>9872074</x:v>
       </x:c>
       <x:c r="C27" s="10" t="str">
-        <x:v>supplement records</x:v>
+        <x:v>Mixed-grain records: 1,889,234 modifications + 7,982,840 monthly activity records; not loans</x:v>
       </x:c>
       <x:c r="D27" s="10" t="str">
-        <x:v>Observed 2022-01–2023-02</x:v>
+        <x:v>14 activity dates: 2022-01–2023-02; modification effective dates 2009–2017</x:v>
       </x:c>
       <x:c r="E27" s="10" t="str">
-        <x:v>Separate loss-mitigation case</x:v>
+        <x:v>Selected HAMP modified-loan workout cohort; aggregate audit only</x:v>
       </x:c>
       <x:c r="F27" s="10" t="str">
-        <x:v>Không thêm Freddie vintage; 2018–2021 coverage chưa established</x:v>
+        <x:v>Treasury lists updates 2018-01–2023-02; local archive has no 2018–2021 activity. Not general PD or Freddie; Not Reported is not default.</x:v>
       </x:c>
       <x:c r="G27" s="10" t="str">
-        <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/TREASURY_HAMP_DATA_REVIEW_VI.md</x:v>
+        <x:v>https://github.com/susayold/credit-atlas/blob/main/docs/TREASURY_HAMP_DATA_REVIEW_VI.md</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="50" customHeight="1">
@@ -3077,10 +3079,10 @@
     </x:row>
     <x:row r="29" ht="50" customHeight="1">
       <x:c r="A29" s="10" t="str">
-        <x:v>NMDB Performance</x:v>
-      </x:c>
-      <x:c r="B29" s="19" t="n">
-        <x:v>261856</x:v>
+        <x:v>NMDB Performance — All geographies</x:v>
+      </x:c>
+      <x:c r="B29" s="19" t="str">
+        <x:v>261,856</x:v>
       </x:c>
       <x:c r="C29" s="10" t="str">
         <x:v>aggregate rows</x:v>
@@ -3089,46 +3091,111 @@
         <x:v>2002Q1–2026Q2</x:v>
       </x:c>
       <x:c r="E29" s="10" t="str">
-        <x:v>P2 market performance context</x:v>
+        <x:v>P2 full-geography performance context</x:v>
       </x:c>
       <x:c r="F29" s="10" t="str">
-        <x:v>13 fields; context khác loan-level outcomes</x:v>
+        <x:v>13 fields; 764 suppressed + 48,028 blank/dot VALUE1; aggregate rates, not loan-level outcomes</x:v>
       </x:c>
       <x:c r="G29" s="10" t="str">
         <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/FHFA_NMDB_AGGREGATE_PERFORMANCE_VI.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="24" customHeight="1">
-      <x:c r="A30" s="2"/>
-      <x:c r="B30" s="2"/>
-      <x:c r="C30" s="2"/>
-      <x:c r="D30" s="2"/>
-      <x:c r="E30" s="2"/>
-      <x:c r="F30" s="2"/>
-      <x:c r="G30" s="2"/>
-    </x:row>
-    <x:row r="31" ht="24" customHeight="1">
-      <x:c r="A31" s="2"/>
-      <x:c r="B31" s="2"/>
-      <x:c r="C31" s="2"/>
-      <x:c r="D31" s="2"/>
-      <x:c r="E31" s="2"/>
-      <x:c r="F31" s="2"/>
-      <x:c r="G31" s="2"/>
+    <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A30" s="10" t="str">
+        <x:v>NMDB Performance — National/census areas</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>25,088 raw / 1,568 national</x:v>
+      </x:c>
+      <x:c r="C30" s="10" t="str">
+        <x:v>aggregate rows</x:v>
+      </x:c>
+      <x:c r="D30" s="10" t="str">
+        <x:v>2002Q1–2026Q2</x:v>
+      </x:c>
+      <x:c r="E30" s="10" t="str">
+        <x:v>P2 national/census-area performance context</x:v>
+      </x:c>
+      <x:c r="F30" s="10" t="str">
+        <x:v>13 fields; latest 2 quarters preliminary; separate from all-geographies and state packages</x:v>
+      </x:c>
+      <x:c r="G30" s="10" t="str">
+        <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/NMDB_PERFORMANCE_CONTEXT_VI.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A31" s="10" t="str">
+        <x:v>NMDB Performance — States</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>79,968</x:v>
+      </x:c>
+      <x:c r="C31" s="10" t="str">
+        <x:v>aggregate rows</x:v>
+      </x:c>
+      <x:c r="D31" s="10" t="str">
+        <x:v>2002Q1–2026Q2</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="str">
+        <x:v>P2 state/DC performance context</x:v>
+      </x:c>
+      <x:c r="F31" s="10" t="str">
+        <x:v>13 fields; state package and route are separate; preserve suppression/missingness; not loan-level PD</x:v>
+      </x:c>
+      <x:c r="G31" s="10" t="str">
+        <x:v>https://github.com/susayold/credit-atlas/blob/b997c20/docs/FHFA_NMDB_STATE_PERFORMANCE_SOURCE_REVIEW_VI.md</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
-      <x:c r="D32" s="2"/>
-      <x:c r="E32" s="2"/>
-      <x:c r="F32" s="2"/>
-      <x:c r="G32" s="2"/>
+      <x:c r="A32" s="2" t="str">
+        <x:v>LendingClub accepted — Mendeley v1</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>1,055,054</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>rows</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>2016Q1–2020Q2</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="str">
+        <x:v>P1 resolved/expired-loan cohort diagnostics</x:v>
+      </x:c>
+      <x:c r="F32" s="2" t="str">
+        <x:v>90 fields; unique id; 838,429 Fully Paid / 216,625 Charged Off; separate from Kaggle snapshot; CC BY 4.0, upstream rights review open</x:v>
+      </x:c>
+      <x:c r="G32" s="2" t="str">
+        <x:v>https://data.mendeley.com/datasets/mvvd3dnfyz/1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>LendingClub issuer field dictionary</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>definitions checked</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>Acquired 2026-10-12</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>P1 source semantics / candidate mapping</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>XLSX definitions do not prove decision-time feature availability; issuer identity and redistribution rights unqualified</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>https://resources.lendingclub.com/LCDataDictionary.xlsx</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2561f4547714159"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae03f439b6e0412c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3279,7 +3346,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a62bdb4297046a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R564a15e76b964773"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh P4 acceptance and plan evidence
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R449a4638e97547c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Rbd2632f7905e4c3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R10b661a2f9a14ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R05c956332bd84737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R8dbe4b0726f14c8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R454a45309e1445bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Ra562ff25b5b7466b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R1319fa384a954a15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -866,10 +866,10 @@
         </x:is>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>Register 123 source records / 17 broad families; P4 Freddie sample UPB is clearly scoped. Excel/JSON downloads now carry local source and artifact lineage; next complete rights, browser/native-Excel parity, and Apple KPI-period mapping.</x:v>
+        <x:v>Register 123 source records / 17 broad families; Freddie 2012 remains a private sample, not owned exposure. P4 XLSX/JSON exports carry source and artifact lineage. Full P4 browser/export acceptance now passes 20 checks; next close native Excel, rights/ownership, Apple KPI-period and remaining route parity. No forecast or estimate without a separate documented method and evidence.</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
-        <x:v>P4 XLSX SourceScope read-back passed with 39/39 upstream hashes and formula scan. Seven JSON export families now carry source receipt/output/lineage hashes and derived receipt SHA-256; 32 focused tests pass. Six targeted Edge checks pass; full browser acceptance blocked by frozen Convergence receipt. Native Excel desktop remains open.</x:v>
+        <x:v>P4 XLSX SourceScope read-back: receipt + four output hashes + 39/39 upstream hashes; formula scan pass. Seven JSON export families carry source/output/lineage and derived-receipt hashes; 32 export tests pass. Full P4 browser/export QA: 20/20 checks, 0 errors; 48 focused tests pass, 5 private-evidence skips. Convergence replay passes on pinned Python 3.12.14 / NumPy 2.5.3 / SciPy 1.18.1; frozen receipt unchanged. Native Excel desktop remains open.</x:v>
       </x:c>
       <x:c r="E19" s="10" t="inlineStr">
         <x:is>
@@ -882,7 +882,7 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>123 records; 22/27 groups bound; 5 dispositions (1 Freddie sample-derived exposure without ownership proof, 3 derived, 1 Ginnie pending). P4 Excel/JSON source provenance implemented; XLSX has 39/39 upstream hashes and JSON receipt/hash envelope is tested across 7 report families (32 tests). These hashes do not authenticate Freddie release/terms, publisher rights, or ownership. Six targeted Edge checks pass; broader browser QA stops pre-browser on “Convergence receipt changed”. Apple is one accession, not a full issuer panel/payment schedule. HAMP gap; 392 NMDB cross-route values match. No forecast/imputation; completion remains 26/50.</x:v>
+        <x:v>123 records; 22/27 groups bound; five explicit dispositions (1 Freddie sample-derived exposure without ownership proof; 3 derived; 1 Ginnie pending). P4 XLSX/JSON lineage is receipt-bound; browser acceptance passes 20 checks, 0 errors. These hashes and UI tests do not authenticate Freddie release/terms, rights, or portfolio ownership. Apple is one accession, not a full issuer panel/payment schedule. HAMP gaps remain missing; no forecast/imputation. Capability completion stays 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="75" customHeight="1">
@@ -1670,7 +1670,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45984e14f57b4865"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0390b6c3e01a4448"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3540,7 +3540,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R021ad61fdac542f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R535e7f5ef2464c6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4644,11 +4644,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R6ecc621862de4511"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R5bbd6ab513634c3f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R227e0aee569a4bf6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c5a7f1f320545e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4853,7 +4853,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02cb401d55694095"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62248312cc824da5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document Apple FY2025 KPI trace and P4 Excel QA
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R8dbe4b0726f14c8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R454a45309e1445bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Ra562ff25b5b7466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R1319fa384a954a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rb1423606e3c74b49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R2b33310d02c54b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Rdb84d4146b164a84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R1da05c9ce4c84a77"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -866,10 +866,10 @@
         </x:is>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>Register 123 source records / 17 broad families; Freddie 2012 remains a private sample, not owned exposure. P4 XLSX/JSON exports carry source and artifact lineage. Full P4 browser/export acceptance now passes 20 checks; next close native Excel, rights/ownership, Apple KPI-period and remaining route parity. No forecast or estimate without a separate documented method and evidence.</x:v>
+        <x:v>N02 binds 22/27 parent groups across 123 source records; five groups have explicit dispositions. Apple FY2025 now has a four-ratio source crosswalk to SEC concepts, accession, period, USD unit and filing date. P4 browser/export passes 20 checks and one source-bound workbook passes Excel desktop. Remaining: other routes, rights/ownership, Apple point-in-time and debt-service qualification. No forecast/imputation.</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
-        <x:v>P4 XLSX SourceScope read-back: receipt + four output hashes + 39/39 upstream hashes; formula scan pass. Seven JSON export families carry source/output/lineage and derived-receipt hashes; 32 export tests pass. Full P4 browser/export QA: 20/20 checks, 0 errors; 48 focused tests pass, 5 private-evidence skips. Convergence replay passes on pinned Python 3.12.14 / NumPy 2.5.3 / SciPy 1.18.1; frozen receipt unchanged. Native Excel desktop remains open.</x:v>
+        <x:v>P4 source-bound XLSX read-back: 7 sheets, 19 formulas, 0 errors, no external links, 39/39 upstream hashes; Excel 16.0 read-only/recalc pass. P4 JSON has source/output/lineage hashes; 32 export tests and 20 browser checks pass, 0 browser errors. Apple ratios: current 0.893292922x; liabilities/assets 79.475338283%; net margin 26.915064122%; OCF/revenue 26.788190148%. Current SEC snapshot is not PIT-qualified; interest coverage unavailable.</x:v>
       </x:c>
       <x:c r="E19" s="10" t="inlineStr">
         <x:is>
@@ -882,7 +882,7 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>123 records; 22/27 groups bound; five explicit dispositions (1 Freddie sample-derived exposure without ownership proof; 3 derived; 1 Ginnie pending). P4 XLSX/JSON lineage is receipt-bound; browser acceptance passes 20 checks, 0 errors. These hashes and UI tests do not authenticate Freddie release/terms, rights, or portfolio ownership. Apple is one accession, not a full issuer panel/payment schedule. HAMP gaps remain missing; no forecast/imputation. Capability completion stays 26/50.</x:v>
+        <x:v>Apple source path is two distinct acquisitions crosswalked by CIK/accession/concept/context; issuer copies are not byte-matched to SEC. Its four ratios are descriptive consolidated-company metrics, not PD/EL/DSCR. Interest expense candidate is missing, so coverage stays unavailable. No historical point-in-time, complete debt schedule or covenant status. Freddie remains sample-only; ownership, rights, other native Excel routes and broader KPI parity remain open. HAMP gaps stay missing. Capability completion stays 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="75" customHeight="1">
@@ -1670,7 +1670,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0390b6c3e01a4448"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07692fbb78154e60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3540,7 +3540,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R535e7f5ef2464c6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R441ace7a56594fc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4644,11 +4644,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R5bbd6ab513634c3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Rbfc8a7b095cc4923"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c5a7f1f320545e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8f58a53ad84dbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4853,7 +4853,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62248312cc824da5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2f4693ad105402a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix NMDB Excel filter and record native acceptance
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rb1423606e3c74b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R2b33310d02c54b27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Rdb84d4146b164a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R1da05c9ce4c84a77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R30bc4c7abe714d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Rb42ee9a346c44524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R671e0ef0dbc14ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R70c848322b9347c3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -885,7 +885,7 @@
         <x:v>Apple source path is two distinct acquisitions crosswalked by CIK/accession/concept/context; issuer copies are not byte-matched to SEC. Its four ratios are descriptive consolidated-company metrics, not PD/EL/DSCR. Interest expense candidate is missing, so coverage stays unavailable. No historical point-in-time, complete debt schedule or covenant status. Freddie remains sample-only; ownership, rights, other native Excel routes and broader KPI parity remain open. HAMP gaps stay missing. Capability completion stays 26/50.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="75" customHeight="1">
+    <x:row r="20" ht="105" customHeight="1">
       <x:c r="A20" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N03</x:t>
@@ -917,7 +917,7 @@
         </x:is>
       </x:c>
       <x:c r="G20" s="17" t="str">
-        <x:v>N03: Full-geography API/UI and filtered Excel pass; 15 tests + 9 Edge checks (100 metros, 98-quarter state trend, suppression). Native Excel and other N03 KPIs remain open.</x:v>
+        <x:v>One VT / Government–Non-Conventional / P3089DL export passes Excel 16.0: 98×12-cell parity, 17 suppressed blanks, 0 formula errors/links; bytes unchanged. Fixed duplicate Table/sheet filter (7 tests pass). Other queries and KPI traces remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="68" customHeight="1">
@@ -1670,7 +1670,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07692fbb78154e60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66c53ba2dfa043a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3540,7 +3540,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R441ace7a56594fc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7c9e81ea26429f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4644,11 +4644,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Rbfc8a7b095cc4923"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R21bfea5356894d97"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8f58a53ad84dbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2da98d6e75a40b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4853,7 +4853,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2f4693ad105402a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra99791e706f945fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify NMDB Excel exports and fix duplicate filters
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R30bc4c7abe714d6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Rb42ee9a346c44524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R671e0ef0dbc14ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R70c848322b9347c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R148ffaddd1634c0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Rc5d370d44d944473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R86f7c24508024faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R5ef204c0db7048a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -917,7 +917,7 @@
         </x:is>
       </x:c>
       <x:c r="G20" s="17" t="str">
-        <x:v>One VT / Government–Non-Conventional / P3089DL export passes Excel 16.0: 98×12-cell parity, 17 suppressed blanks, 0 formula errors/links; bytes unchanged. Fixed duplicate Table/sheet filter (7 tests pass). Other queries and KPI traces remain open.</x:v>
+        <x:v>Excel 16 read-only: performance suppression query 98×12; New AVE_INTRATE 28×18; Outstanding PCT_MTMLTV_GT100 54×18. Suppressed values stay blank; filters work. Other queries/KPI traces remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="68" customHeight="1">
@@ -953,7 +953,7 @@
       </x:c>
       <x:c r="G21" s="17" t="str"/>
     </x:row>
-    <x:row r="22" ht="75" customHeight="1">
+    <x:row r="22" ht="105" customHeight="1">
       <x:c r="A22" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N05</x:t>
@@ -984,13 +984,11 @@
           <x:t xml:space="preserve">Đang làm</x:t>
         </x:is>
       </x:c>
-      <x:c r="G22" s="17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">New/Outstanding mart/API rechecked: 3.04M annual and 535,464 quarterly rows; key, weighting and missingness checks pass. 8 representative browser/filter/XLSX checks; full routes and native Excel open.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="75" customHeight="1">
+      <x:c r="G22" s="17" t="str">
+        <x:v>FHFA release-bound mart: 3.04M annual + 535,464 quarterly rows. Excel 16 parity passes New AVE_INTRATE (28/28) and Outstanding PCT_MTMLTV_GT100 (54/54); no imputation. Broader query coverage remains open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="105" customHeight="1">
       <x:c r="A23" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N06</x:t>
@@ -1021,10 +1019,8 @@
           <x:t xml:space="preserve">Đang làm</x:t>
         </x:is>
       </x:c>
-      <x:c r="G23" s="17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8 Edge checks pass for filters, VALUE1/VALUE2, suppression/null and query-scoped XLSX. Remaining geography/market/period cases and native Excel open.</x:t>
-        </x:is>
+      <x:c r="G23" s="17" t="str">
+        <x:v>D02 state reference: 79,968 ×13 source rows match; 68 suppressed rows and 14,535 blank rates retained. Excel 16 opens the 24-sheet workbook; Table filter visible; bytes unchanged. Other routes/filters remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="75" customHeight="1">
@@ -1472,7 +1468,7 @@
       </x:c>
       <x:c r="G36" s="17" t="str"/>
     </x:row>
-    <x:row r="37" ht="75" customHeight="1">
+    <x:row r="37" ht="105" customHeight="1">
       <x:c r="A37" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N20</x:t>
@@ -1503,10 +1499,8 @@
           <x:t xml:space="preserve">Đang làm</x:t>
         </x:is>
       </x:c>
-      <x:c r="G37" s="17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">HMDA, PUDB, NMDB and ABS Excel packages exist; representative browser/export checks pass. Native Excel desktop recalculation and remaining route parity open.</x:t>
-        </x:is>
+      <x:c r="G37" s="17" t="str">
+        <x:v>Excel 16 read-only passes: plan workbook, one performance query, two New/Outstanding exports and the 24-sheet D02 state reference. NMDB source values and suppression stay intact; remaining HMDA/PUDB/HUD routes and broader filters need QA.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="68" customHeight="1">
@@ -1670,7 +1664,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66c53ba2dfa043a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4888865b27d041dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3540,7 +3534,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7c9e81ea26429f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R936890094a8d422e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4644,11 +4638,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R21bfea5356894d97"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R678f20b49d104bcd"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2da98d6e75a40b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36c130dce6a4747"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4853,7 +4847,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra99791e706f945fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9070d03b99e64b47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh plan with current HMDA evidence
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R148ffaddd1634c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Rc5d370d44d944473"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R86f7c24508024faa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R5ef204c0db7048a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R6869e96fa8c8424d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R02a9638b2c6f420c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R28076d0c51b946b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R88247f5426d345eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -882,10 +882,10 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>Apple source path is two distinct acquisitions crosswalked by CIK/accession/concept/context; issuer copies are not byte-matched to SEC. Its four ratios are descriptive consolidated-company metrics, not PD/EL/DSCR. Interest expense candidate is missing, so coverage stays unavailable. No historical point-in-time, complete debt schedule or covenant status. Freddie remains sample-only; ownership, rights, other native Excel routes and broader KPI parity remain open. HAMP gaps stay missing. Capability completion stays 26/50.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="105" customHeight="1">
+        <x:v>HMDA current-code browser QA: 46 checks, receipt app.js hashes match current code, zero page/console errors; all nine release-bound workbooks pass Excel 16.0 read-only/recalc (177 formulas, zero errors/links); 146 HMDA tests pass. Release comparability and reuse rights remain open. Apple remains one descriptive accession without point-in-time/debt-service qualification; Freddie stays a private sample, not owned exposure; HAMP gaps remain missing. No forecast; capability stays 26/50.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="202.5" customHeight="1">
       <x:c r="A20" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N03</x:t>
@@ -917,7 +917,7 @@
         </x:is>
       </x:c>
       <x:c r="G20" s="17" t="str">
-        <x:v>Excel 16 read-only: performance suppression query 98×12; New AVE_INTRATE 28×18; Outstanding PCT_MTMLTV_GT100 54×18. Suppressed values stay blank; filters work. Other queries/KPI traces remain open.</x:v>
+        <x:v>NMDB Excel 16 read-only: performance suppression query 98×12; New AVE_INTRATE 28×18; Outstanding PCT_MTMLTV_GT100 54×18. HMDA fixed-2023-mix raw-source audit passes 70/70 checks for mart, attrition, denominators/amounts, reference/common-support weights, missing strata and hash stability. This verifies local calculations only, not risk prediction/fairness/causality. Remaining N03 KPI and release comparability/rights work stays open; no forecast; 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="68" customHeight="1">
@@ -1664,7 +1664,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4888865b27d041dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4348e26ced734ddb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3534,7 +3534,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R936890094a8d422e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e21244e1424498b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4638,11 +4638,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R678f20b49d104bcd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R33f1780029ea41d7"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36c130dce6a4747"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41661eaa804b4819"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4847,7 +4847,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9070d03b99e64b47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6af7107e48494b69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document HMDA release comparability audit
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R6869e96fa8c8424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R02a9638b2c6f420c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R28076d0c51b946b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R88247f5426d345eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rc4b76a3944614bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R974631f1fb0d496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R50bd4a1d62764c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R8e864f5ce77c40ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -854,7 +854,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="19" ht="224.39999389648438" hidden="0" customHeight="1">
+    <x:row r="19" ht="225" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N02</x:t>
@@ -882,7 +882,7 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>HMDA current-code browser QA: 46 checks, receipt app.js hashes match current code, zero page/console errors; all nine release-bound workbooks pass Excel 16.0 read-only/recalc (177 formulas, zero errors/links); 146 HMDA tests pass. Release comparability and reuse rights remain open. Apple remains one descriptive accession without point-in-time/debt-service qualification; Freddie stays a private sample, not owned exposure; HAMP gaps remain missing. No forecast; capability stays 26/50.</x:v>
+        <x:v>HMDA: official Data Browser mapping is 2018–22 Three-Year, 2023–24 One-Year, 2025 Snapshot. The app’s 2019 One-Year archive is distinct from Browser 2019 Three-Year. Receipt-bound same-year 2025 audit: Snapshot 13,543,606 rows/4,782 reporters vs Dynamic 13,558,306/4,794; +14,700 rows, +12 reporters, denied share −0.02304073 pp. No explicit raw redistribution license found on reviewed product pages; keep raw private pending publisher-specific rights confirmation. Release/year parity and KPI lineage remain open; HMDA is not repayment/default performance. No forecast; 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="202.5" customHeight="1">
@@ -1664,7 +1664,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4348e26ced734ddb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbc811e3fade44ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3534,7 +3534,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e21244e1424498b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c69109213dd4446"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4638,11 +4638,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R33f1780029ea41d7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Rf8afb264250046e9"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41661eaa804b4819"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1da1428878094b0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4847,7 +4847,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6af7107e48494b69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab0f34daf2be4e57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add HMDA Browser release audit workbook and plan
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rc4b76a3944614bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R974631f1fb0d496c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R50bd4a1d62764c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R8e864f5ce77c40ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R4f34e15cfa9c495a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R89c8f903c90741d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Rc007b0d7cd644edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="Rff2a23ec4fde4f99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -854,7 +854,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="19" ht="225" hidden="0" customHeight="1">
+    <x:row r="19" ht="262.5" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N02</x:t>
@@ -882,7 +882,7 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>HMDA: official Data Browser mapping is 2018–22 Three-Year, 2023–24 One-Year, 2025 Snapshot. The app’s 2019 One-Year archive is distinct from Browser 2019 Three-Year. Receipt-bound same-year 2025 audit: Snapshot 13,543,606 rows/4,782 reporters vs Dynamic 13,558,306/4,794; +14,700 rows, +12 reporters, denied share −0.02304073 pp. No explicit raw redistribution license found on reviewed product pages; keep raw private pending publisher-specific rights confirmation. Release/year parity and KPI lineage remain open; HMDA is not repayment/default performance. No forecast; 26/50.</x:v>
+        <x:v>HMDA: official Browser action-count API audit 2018–25 passes (8 years). Exact same-vintage local receipt matches: 2018 Three-Year and 2023–25 (4); 2019–22 app One-Year archives differ from Browser Three-Year. Three-Year minus One-Year row deltas: +10,763/+32,298/+42,616/+26,668; denied-share deltas: +0.00422048/−0.01064505/+0.10251269/+0.14468237 pp. These are aggregate release-state deltas, with no row matching or borrower-performance meaning. The 2025 Snapshot/Dynamic audit is separate. No explicit raw redistribution license found on reviewed product pages; raw remains private. Rights, dimensional parity and KPI lineage stay open; no forecast; 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="202.5" customHeight="1">
@@ -1664,7 +1664,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbc811e3fade44ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc587503accb84fa2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3534,7 +3534,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c69109213dd4446"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc143a67191c744c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4638,11 +4638,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Rf8afb264250046e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R498d03c2a6534326"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1da1428878094b0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R056b50e38c044953"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4847,7 +4847,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab0f34daf2be4e57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3c3e71b34934abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add filtered HMDA Excel intersection export
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rf0560c8b794d4480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R7fc579239f8849e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Rf5b2d27bdb4f4abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="Rb1248f289a5b4bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R83cae44ad3a045e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R4f30fcdaf5ef4241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R53c9eab6ba3e4c68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="Re22db09957bc4ee5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -852,7 +852,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="19" ht="292.5" hidden="0" customHeight="1">
+    <x:row r="19" ht="322.5" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N02</x:t>
@@ -880,7 +880,7 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>HMDA Browser API: 8 years pass; 4 same-vintage exact local matches (2018, 2023–25); 2019–22 One-Year vs Three-Year remain aggregate-only (see report). 2025 Snapshot: 5 filtered API profiles match local; 4 app marginals + CA × conventional intersection match API. Snapshot + Dynamic smoke each pass KPI/URL/JSON; Dynamic API parity, older annual panels and filtered XLSX remain open. Six-sheet Excel audit: 124 formulas, Excel 16 PASS. Raw rights unconfirmed/private; broader intersections, harmonization and KPI lineage open. No forecast; 26/50.</x:v>
+        <x:v>HMDA Browser API: 8 years pass; 4 same-vintage exact local matches (2018, 2023–25); 2019–22 One-Year vs Three-Year remain aggregate-only. Snapshot: five filtered API scopes match local; four marginals + CA × conventional intersection match API. Snapshot and Dynamic 2025 each pass 5 browser checks (KPI/URL/JSON/XLSX); both filtered workbooks pass Excel 16 with 12 formulas, 4/4 reconciliation checks, zero errors/links, unchanged bytes. Independent API/raw parity remains Snapshot-only. Dynamic official API parity and older annual panels remain open. Raw reuse rights, broader intersections, harmonization and KPI lineage remain open. No forecast; 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="202.5" customHeight="1">
@@ -1662,7 +1662,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ce9c99045824351"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7d52a96e13f49c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3532,7 +3532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf77179c3e6694953"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e55dba0bcd242f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4636,11 +4636,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R061b31dccb864afa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R53fd4e3b2a4a4cc0"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde39580e24834c88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8cb2404e3c14b1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4845,7 +4845,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11bdee80966748d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfe3495df034273"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update HMDA plan and validation evidence
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R83cae44ad3a045e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R4f30fcdaf5ef4241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R53c9eab6ba3e4c68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="Re22db09957bc4ee5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R439b856ff9ac4ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R490b72bf4a5040fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R5929cd531f7d42d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R86cbdaf6cacd43e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -880,7 +880,7 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>HMDA Browser API: 8 years pass; 4 same-vintage exact local matches (2018, 2023–25); 2019–22 One-Year vs Three-Year remain aggregate-only. Snapshot: five filtered API scopes match local; four marginals + CA × conventional intersection match API. Snapshot and Dynamic 2025 each pass 5 browser checks (KPI/URL/JSON/XLSX); both filtered workbooks pass Excel 16 with 12 formulas, 4/4 reconciliation checks, zero errors/links, unchanged bytes. Independent API/raw parity remains Snapshot-only. Dynamic official API parity and older annual panels remain open. Raw reuse rights, broader intersections, harmonization and KPI lineage remain open. No forecast; 26/50.</x:v>
+        <x:v>HMDA Browser API: 8 years pass; 4 same-vintage exact local matches (2018, 2023–25); 2019–22 One-Year vs Three-Year remain aggregate-only. Snapshot: five filtered API scopes match local; four marginals + CA × conventional intersection match API. Snapshot and Dynamic 2025 each pass 5 browser checks (KPI/URL/JSON/XLSX); both filtered workbooks pass Excel 16 with 12 formulas, 4/4 reconciliation checks, zero errors/links, unchanged bytes. Independent API/raw parity applies to Snapshot. Prior 2018–2024 panel receipts pass (2018/2019 4+4; 2020–24 suite 21 total incl. 15 panel-specific); current broad replay stopped before browser, annual render code unchanged. Dynamic is separate weekly S3, not a Browser API target; 18/10 HEAD metadata matches 10/11 capture and local hashes match receipts. Raw rights, broader intersections, harmonization and KPI lineage remain open. No forecast; 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="202.5" customHeight="1">
@@ -1662,7 +1662,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7d52a96e13f49c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcab2e9d71fed4769"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3532,7 +3532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e55dba0bcd242f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f97a4ce7684453"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4636,11 +4636,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R53fd4e3b2a4a4cc0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R5a888f5343ba418f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8cb2404e3c14b1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ca4cf4ce7b54df9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4845,7 +4845,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfe3495df034273"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31c3c7a0af744f25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Extend NMDB query-grid acceptance
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R439b856ff9ac4ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R490b72bf4a5040fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R5929cd531f7d42d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R86cbdaf6cacd43e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R679d0d3b4b634822"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R2fe9f6592156400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R2d2ceff0c72642b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R7560eafa27904492"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -951,7 +951,7 @@
       </x:c>
       <x:c r="G21" s="17" t="str"/>
     </x:row>
-    <x:row r="22" ht="105" customHeight="1">
+    <x:row r="22" ht="132" hidden="0" customHeight="1">
       <x:c r="A22" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N05</x:t>
@@ -983,10 +983,10 @@
         </x:is>
       </x:c>
       <x:c r="G22" s="17" t="str">
-        <x:v>FHFA release-bound mart: 3.04M annual + 535,464 quarterly rows. Excel 16 parity passes New AVE_INTRATE (28/28) and Outstanding PCT_MTMLTV_GT100 (54/54); no imputation. Broader query coverage remains open.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="105" customHeight="1">
+        <x:v>FHFA receipt-bound mart: New 3,038,100 annual + Outstanding 535,464 quarterly rows. API grid: 235 scopes; all 115 New + 68 Outstanding series/weight pairs, 31 market categories and five geography levels per product; source keys, weights, units, suppression/null and no-imputation checks retained. Flow and active-stock remain separate. Broad matrix, not every Cartesian filter; no PD/model claim.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A23" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N06</x:t>
@@ -1018,7 +1018,7 @@
         </x:is>
       </x:c>
       <x:c r="G23" s="17" t="str">
-        <x:v>D02 state reference: 79,968 ×13 source rows match; 68 suppressed rows and 14,535 blank rates retained. Excel 16 opens the 24-sheet workbook; Table filter visible; bytes unchanged. Other routes/filters remain open.</x:v>
+        <x:v>Filtered API/XLSX grid: 56 exports, 1,758 rows × 18 = 31,644 cells match API. Covers all market categories/geography levels, period edges and selected VALUE2. Alaska State × Jumbo preserves seven suppressed rows as unavailable. Browser: 8/8, no errors, 390px fits. Excel 16.0 read-only/full-rebuild: New Alaska/Jumbo 27×18 and Outstanding VALUE2 54×18; table filters/charts, 0 formulas/errors/external links, bytes unchanged. Full Cartesian/native coverage remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="75" customHeight="1">
@@ -1662,7 +1662,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcab2e9d71fed4769"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a62caaab07431e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3532,7 +3532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f97a4ce7684453"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae56fa18ee9a4f7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4636,11 +4636,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R5a888f5343ba418f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Rf2423548f1df4195"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ca4cf4ce7b54df9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re677347cd00445ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4845,7 +4845,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31c3c7a0af744f25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0936bddd7b1f4a25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add reciprocal project source lineage
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="R679d0d3b4b634822"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R2fe9f6592156400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R2d2ceff0c72642b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R7560eafa27904492"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rbb9030f3e67b42dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R25024366001d453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R170d7b39222d4fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R07bbf1d23cdc428a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -815,7 +815,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18" ht="68" customHeight="1">
+    <x:row r="18" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A18" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N01</x:t>
@@ -836,23 +836,19 @@
           <x:t xml:space="preserve">Ledger hiện tại</x:t>
         </x:is>
       </x:c>
-      <x:c r="E18" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Tổng 26/50 tái tạo từ ledger; UI/docs không gọi 52% là D01; historical labels được giữ</x:t>
-        </x:is>
+      <x:c r="E18" s="9" t="str">
+        <x:v>Tổng 26/50 tái tạo từ ledger P1–P5; D01 được theo dõi riêng theo R0–R4. Current UI/docs tách hai scope; legacy checkpoints cần correction note.</x:v>
       </x:c>
       <x:c r="F18" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Đang làm</x:t>
         </x:is>
       </x:c>
-      <x:c r="G18" s="17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">API/UI derives P1-P5 from the ledger; final local runtime review remains.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="322.5" hidden="0" customHeight="1">
+      <x:c r="G18" s="17" t="str">
+        <x:v>API/static runtime PASS (12 checks): 27 dataset groups, 123 source records, 15 method cards; 15/15 source-linked with 50 reciprocal links across 33 source rows. Ledger remains 26/50; D01 gates are separate. Browser rendering and stale-label scan remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N02</x:t>
@@ -869,10 +865,8 @@
       <x:c r="D19" s="10" t="str">
         <x:v>P4 source-bound XLSX read-back: 7 sheets, 19 formulas, 0 errors, no external links, 39/39 upstream hashes; Excel 16.0 read-only/recalc pass. P4 JSON has source/output/lineage hashes; 32 export tests and 20 browser checks pass, 0 browser errors. Apple ratios: current 0.893292922x; liabilities/assets 79.475338283%; net margin 26.915064122%; OCF/revenue 26.788190148%. Current SEC snapshot is not PIT-qualified; interest coverage unavailable.</x:v>
       </x:c>
-      <x:c r="E19" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">27 groups statused; each KPI traces source → field → filter → formula → API/Excel; rights resolved/fenced; no unsupported estimates.</x:t>
-        </x:is>
+      <x:c r="E19" s="10" t="str">
+        <x:v>27 groups have explicit disposition; 22/27 have source-object records. Method/source: 15/15 cards, 50 reciprocal links across 33/123 source records. Five groups remain classified; validate source → field → KPI and rights.</x:v>
       </x:c>
       <x:c r="F19" s="17" t="inlineStr">
         <x:is>
@@ -880,10 +874,10 @@
         </x:is>
       </x:c>
       <x:c r="G19" s="17" t="str">
-        <x:v>HMDA Browser API: 8 years pass; 4 same-vintage exact local matches (2018, 2023–25); 2019–22 One-Year vs Three-Year remain aggregate-only. Snapshot: five filtered API scopes match local; four marginals + CA × conventional intersection match API. Snapshot and Dynamic 2025 each pass 5 browser checks (KPI/URL/JSON/XLSX); both filtered workbooks pass Excel 16 with 12 formulas, 4/4 reconciliation checks, zero errors/links, unchanged bytes. Independent API/raw parity applies to Snapshot. Prior 2018–2024 panel receipts pass (2018/2019 4+4; 2020–24 suite 21 total incl. 15 panel-specific); current broad replay stopped before browser, annual render code unchanged. Dynamic is separate weekly S3, not a Browser API target; 18/10 HEAD metadata matches 10/11 capture and local hashes match receipts. Raw rights, broader intersections, harmonization and KPI lineage remain open. No forecast; 26/50.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="202.5" customHeight="1">
+        <x:v>N02 lineage: D01 → Freddie; UCI 350/365 → UCI source and metadata; P4 → Freddie upstream sample-derived UPB only (not owned portfolio); Toyota/Nissan filings → recovery studies and the 103-period ABS finding. LendingClub now has three valid evidence documents. Still open: five group dispositions, Freddie release/rights, and KPI-to-field/output parity. 90 source records without method-card links are not presumed invalid.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="132" hidden="0" customHeight="1">
       <x:c r="A20" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N03</x:t>
@@ -904,10 +898,8 @@
           <x:t xml:space="preserve">N02, model/scenario artifacts</x:t>
         </x:is>
       </x:c>
-      <x:c r="E20" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Từng output số đi tới method/input; phân biệt publisher-imputed với app-imputed; không sửa frozen studies</x:t>
-        </x:is>
+      <x:c r="E20" s="9" t="str">
+        <x:v>15/15 cards have target, method, validation, limits, valid evidence paths and reciprocal source-release links. Still map each material KPI/output to exact fields, filters, units, code and assumptions; distinguish publisher/app imputation.</x:v>
       </x:c>
       <x:c r="F20" s="17" t="inlineStr">
         <x:is>
@@ -915,7 +907,7 @@
         </x:is>
       </x:c>
       <x:c r="G20" s="17" t="str">
-        <x:v>NMDB Excel 16 read-only: performance suppression query 98×12; New AVE_INTRATE 28×18; Outstanding PCT_MTMLTV_GT100 54×18. HMDA fixed-2023-mix raw-source audit passes 70/70 checks for mart, attrition, denominators/amounts, reference/common-support weights, missing strata and hash stability. This verifies local calculations only, not risk prediction/fairness/causality. Remaining N03 KPI and release comparability/rights work stays open; no forecast; 26/50.</x:v>
+        <x:v>Focused tests: 10 passed; API/static + lineage acceptance: 12/12. 50 reciprocal method ↔ source links across 33 source rows; LendingClub broken evidence path fixed. P4 explicitly says Freddie is upstream sample-derived UPB only. N03 remains open until material numeric outputs, units and assumptions trace through code and source data; ledger stays 26/50.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="68" customHeight="1">
@@ -1662,7 +1654,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a62caaab07431e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a32b11495584a7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3532,7 +3524,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae56fa18ee9a4f7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe00ec7247a64ff1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4636,11 +4628,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Rf2423548f1df4195"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R0fca97ff7ef14f1d"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re677347cd00445ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27e8b718a1d3415b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4845,7 +4837,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0936bddd7b1f4a25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829a25f4d9954784"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify CreditAtlas completion scope in research plan
</commit_message>
<xml_diff>
--- a/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
+++ b/docs/reviews/CreditAtlas-Review-Next-Plan-2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rbb9030f3e67b42dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="R25024366001d453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="R170d7b39222d4fbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="R07bbf1d23cdc428a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ke hoach" sheetId="1" r:id="Rc2ca77fc017442b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 yeu cau" sheetId="2" r:id="Redc96270fd3a41f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Du lieu" sheetId="3" r:id="Rc18b41b71ba14a9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phuong phap" sheetId="4" r:id="Rebaa40223dbc4e7f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -815,7 +815,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="18" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A18" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">N01</x:t>
@@ -837,7 +837,7 @@
         </x:is>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>Tổng 26/50 tái tạo từ ledger P1–P5; D01 được theo dõi riêng theo R0–R4. Current UI/docs tách hai scope; legacy checkpoints cần correction note.</x:v>
+        <x:v>26/50 là ledger toàn CreditAtlas P1–P5; D01 được theo dõi riêng theo R0–R4. UI/docs phân biệt scope; static stale-label scan PASS; browser render trên UI thật vẫn mở.</x:v>
       </x:c>
       <x:c r="F18" s="17" t="inlineStr">
         <x:is>
@@ -845,7 +845,7 @@
         </x:is>
       </x:c>
       <x:c r="G18" s="17" t="str">
-        <x:v>API/static runtime PASS (12 checks): 27 dataset groups, 123 source records, 15 method cards; 15/15 source-linked with 50 reciprocal links across 33 source rows. Ledger remains 26/50; D01 gates are separate. Browser rendering and stale-label scan remain open.</x:v>
+        <x:v>API/static runtime PASS (12 checks): 27 dataset groups, 123 source records, 15 method cards, 50 capability rows; 26/50, domain counts and D01 R0–R4 reconcile. Fixed register init fallback. Static stale-label scan PASS: 195 Markdown files, 14 D01/ledger co-mentions reviewed, zero false D01 completion claims. Browser UI render is still unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="171.60000610351562" hidden="0" customHeight="1">
@@ -1654,7 +1654,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a32b11495584a7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc544f458b6944e8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3524,7 +3524,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe00ec7247a64ff1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88e079de10784372"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4628,11 +4628,11 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R0fca97ff7ef14f1d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R114f1a6de7af4bed"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27e8b718a1d3415b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9230a415d154c7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4837,7 +4837,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829a25f4d9954784"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ae33a94596d4d99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>